<commit_message>
MPOs/off-prem: refresh Lytt POS Items Pics photo feed (Report_43 / Promos_Report_5)
Overwrote lytt_pos_displays.xlsx and lytt_pos_promos.xlsx with the new
iSellBeer exports and reran generate_lytt_pos.py.

  82 -> 87 photo-bearing rows, 32 -> 37 distinct photos
  Displays 74 -> 75 rows, Promos 1 -> 5 rows
  Pablo Lopez 1 -> 6 distinct pics; every other rep unchanged

No new PODS export in this batch, so lytt_pos_pods.xlsx (7 photo rows)
is carried over from the last refresh. No rep is at the 8-pic target yet
(Javier Melo and Dave Ehlers lead at 7).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S5qkVoHxgNnGYvzsGuLGTd
</commit_message>
<xml_diff>
--- a/MPOs/off-prem/lytt_pos_promos.xlsx
+++ b/MPOs/off-prem/lytt_pos_promos.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="62">
   <si>
     <t>Values were filtered by:</t>
   </si>
@@ -23,91 +23,172 @@
     <t>Brands</t>
   </si>
   <si>
+    <t>LYTT BLUE RASPBERRY, LYTT PEACH MANGO</t>
+  </si>
+  <si>
+    <t>Start Date</t>
+  </si>
+  <si>
+    <t>08/01/2026</t>
+  </si>
+  <si>
+    <t>End Date</t>
+  </si>
+  <si>
+    <t>08/20/2026</t>
+  </si>
+  <si>
+    <t>Date/Time</t>
+  </si>
+  <si>
+    <t>Promo #</t>
+  </si>
+  <si>
+    <t>Photo taker</t>
+  </si>
+  <si>
+    <t>District Manager</t>
+  </si>
+  <si>
+    <t>Sales Manager</t>
+  </si>
+  <si>
+    <t>Photo taker's role</t>
+  </si>
+  <si>
+    <t>Promotion type</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>DBA</t>
+  </si>
+  <si>
+    <t>Account #</t>
+  </si>
+  <si>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>Theme</t>
+  </si>
+  <si>
+    <t>Elements</t>
+  </si>
+  <si>
+    <t>Brand</t>
+  </si>
+  <si>
+    <t>Supplier</t>
+  </si>
+  <si>
+    <t>Photo</t>
+  </si>
+  <si>
+    <t>08/19/2026 04:09 PM</t>
+  </si>
+  <si>
+    <t>1.1</t>
+  </si>
+  <si>
+    <t>Pablo Lopez</t>
+  </si>
+  <si>
+    <t>Denise Montes</t>
+  </si>
+  <si>
+    <t>Ashley Furman</t>
+  </si>
+  <si>
+    <t>Sales Rep</t>
+  </si>
+  <si>
+    <t>Feature Activation</t>
+  </si>
+  <si>
+    <t>RONNY'S LIQRS (Z)</t>
+  </si>
+  <si>
+    <t>20114</t>
+  </si>
+  <si>
+    <t>389 MADISON AVENUE</t>
+  </si>
+  <si>
+    <t>PATERSON</t>
+  </si>
+  <si>
+    <t>MBO</t>
+  </si>
+  <si>
+    <t>Poster</t>
+  </si>
+  <si>
     <t>LYTT PEACH MANGO</t>
   </si>
   <si>
-    <t>Start Date</t>
-  </si>
-  <si>
-    <t>08/01/2026</t>
-  </si>
-  <si>
-    <t>End Date</t>
-  </si>
-  <si>
-    <t>08/19/2026</t>
-  </si>
-  <si>
-    <t>Date/Time</t>
-  </si>
-  <si>
-    <t>Promo #</t>
-  </si>
-  <si>
-    <t>Photo taker</t>
-  </si>
-  <si>
-    <t>District Manager</t>
-  </si>
-  <si>
-    <t>Sales Manager</t>
-  </si>
-  <si>
-    <t>Photo taker's role</t>
-  </si>
-  <si>
-    <t>Promotion type</t>
-  </si>
-  <si>
-    <t>Quantity</t>
-  </si>
-  <si>
-    <t>DBA</t>
-  </si>
-  <si>
-    <t>Account #</t>
-  </si>
-  <si>
-    <t>Address</t>
-  </si>
-  <si>
-    <t>City</t>
-  </si>
-  <si>
-    <t>Theme</t>
-  </si>
-  <si>
-    <t>Elements</t>
-  </si>
-  <si>
-    <t>Brand</t>
-  </si>
-  <si>
-    <t>Supplier</t>
-  </si>
-  <si>
-    <t>Photo</t>
+    <t>BOSTON BEER COMPANY</t>
+  </si>
+  <si>
+    <t>08/19/2026 04:08 PM</t>
+  </si>
+  <si>
+    <t>2.1</t>
+  </si>
+  <si>
+    <t>POS</t>
+  </si>
+  <si>
+    <t>08/19/2026 02:11 PM</t>
+  </si>
+  <si>
+    <t>3.1</t>
+  </si>
+  <si>
+    <t>SUNNY'S LIQS.(P)</t>
+  </si>
+  <si>
+    <t>27066</t>
+  </si>
+  <si>
+    <t>413 MONROE ST</t>
+  </si>
+  <si>
+    <t>PASSAIC</t>
+  </si>
+  <si>
+    <t>Poster, POS</t>
+  </si>
+  <si>
+    <t>LYTT BLUE RASPBERRY</t>
+  </si>
+  <si>
+    <t>08/19/2026 01:29 PM</t>
+  </si>
+  <si>
+    <t>4.1</t>
+  </si>
+  <si>
+    <t>REGALADO LIQ</t>
+  </si>
+  <si>
+    <t>26014</t>
+  </si>
+  <si>
+    <t>168 MARKET ST</t>
+  </si>
+  <si>
+    <t>Signage, Window Sign</t>
   </si>
   <si>
     <t>08/13/2026 01:22 PM</t>
   </si>
   <si>
-    <t>1.1</t>
-  </si>
-  <si>
-    <t>Pablo Lopez</t>
-  </si>
-  <si>
-    <t>Denise Montes</t>
-  </si>
-  <si>
-    <t>Ashley Furman</t>
-  </si>
-  <si>
-    <t>Sales Rep</t>
-  </si>
-  <si>
-    <t>Feature Activation</t>
+    <t>5.1</t>
   </si>
   <si>
     <t>FLORIDA DRUGS (A)</t>
@@ -119,16 +200,7 @@
     <t>507 BROADWAY</t>
   </si>
   <si>
-    <t>PATERSON</t>
-  </si>
-  <si>
-    <t>MBO</t>
-  </si>
-  <si>
     <t>Wrap, Poster</t>
-  </si>
-  <si>
-    <t>BOSTON BEER COMPANY</t>
   </si>
 </sst>
 </file>
@@ -525,7 +597,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:Q6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="21.7109375" customWidth="1"/>
@@ -537,12 +609,11 @@
     <col min="8" max="8" width="10.7109375" customWidth="1"/>
     <col min="9" max="9" width="19.7109375" customWidth="1"/>
     <col min="10" max="10" width="11.7109375" customWidth="1"/>
-    <col min="11" max="11" width="14.7109375" customWidth="1"/>
+    <col min="11" max="11" width="20.7109375" customWidth="1"/>
     <col min="12" max="12" width="10.7109375" customWidth="1"/>
     <col min="13" max="13" width="7.7109375" customWidth="1"/>
-    <col min="14" max="14" width="14.7109375" customWidth="1"/>
-    <col min="15" max="15" width="18.7109375" customWidth="1"/>
-    <col min="16" max="16" width="21.7109375" customWidth="1"/>
+    <col min="14" max="14" width="22.7109375" customWidth="1"/>
+    <col min="15" max="16" width="21.7109375" customWidth="1"/>
     <col min="17" max="17" width="7.7109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -643,18 +714,234 @@
         <v>36</v>
       </c>
       <c r="O2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17">
+      <c r="A3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H3" s="2">
+        <v>1</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="P3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q3" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17">
+      <c r="A4" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" s="2">
+        <v>1</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="O4" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="P4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q4" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17">
+      <c r="A5" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H5" s="2">
         <v>2</v>
       </c>
-      <c r="P2" s="2" t="s">
+      <c r="I5" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="O5" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="P5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q5" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17">
+      <c r="A6" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H6" s="2">
+        <v>1</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="O6" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="P6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q6" s="3" t="s">
         <v>23</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="Q2" r:id="rId1"/>
+    <hyperlink ref="Q3" r:id="rId2"/>
+    <hyperlink ref="Q4" r:id="rId3"/>
+    <hyperlink ref="Q5" r:id="rId4"/>
+    <hyperlink ref="Q6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>